<commit_message>
correct name for 1905 Nußdorf und Kahlenbergdorf
</commit_message>
<xml_diff>
--- a/vienna/gr2025/mapping_graetzl_sprengel_wien2025.xlsx
+++ b/vienna/gr2025/mapping_graetzl_sprengel_wien2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\apariihaslacher\repos\austrian-neighbourhood-maps\_intern_Wien-2025\data_final\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\apariihaslacher\repos\austrian-neighbourhood-maps\vienna\gr2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{005B266B-7B9B-4920-9F95-07F8D48EBC69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A65955C-752A-471B-A6E4-C9F3572EAF81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15620" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="mapping" sheetId="1" r:id="rId1"/>
@@ -351,9 +351,6 @@
     <t>Heiligenstadt</t>
   </si>
   <si>
-    <t>Nußdorf-Kahlenbergergdorf</t>
-  </si>
-  <si>
     <t>Neustift am Walde</t>
   </si>
   <si>
@@ -475,6 +472,9 @@
   </si>
   <si>
     <t>has, 06.03.2024</t>
+  </si>
+  <si>
+    <t>Nußdorf und Kahlenbergergdorf</t>
   </si>
 </sst>
 </file>
@@ -860,17 +860,17 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -15043,7 +15043,7 @@
     </row>
     <row r="1017" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1017" t="s">
-        <v>105</v>
+        <v>146</v>
       </c>
       <c r="B1017">
         <v>1905</v>
@@ -15057,7 +15057,7 @@
     </row>
     <row r="1018" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1018" t="s">
-        <v>105</v>
+        <v>146</v>
       </c>
       <c r="B1018">
         <v>1905</v>
@@ -15071,7 +15071,7 @@
     </row>
     <row r="1019" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1019" t="s">
-        <v>105</v>
+        <v>146</v>
       </c>
       <c r="B1019">
         <v>1905</v>
@@ -15085,7 +15085,7 @@
     </row>
     <row r="1020" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1020" t="s">
-        <v>105</v>
+        <v>146</v>
       </c>
       <c r="B1020">
         <v>1905</v>
@@ -15099,7 +15099,7 @@
     </row>
     <row r="1021" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1021" t="s">
-        <v>105</v>
+        <v>146</v>
       </c>
       <c r="B1021">
         <v>1905</v>
@@ -15113,7 +15113,7 @@
     </row>
     <row r="1022" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1022" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B1022">
         <v>1906</v>
@@ -15127,7 +15127,7 @@
     </row>
     <row r="1023" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1023" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B1023">
         <v>1906</v>
@@ -15141,7 +15141,7 @@
     </row>
     <row r="1024" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1024" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B1024">
         <v>1906</v>
@@ -15155,7 +15155,7 @@
     </row>
     <row r="1025" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1025" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B1025">
         <v>1906</v>
@@ -15169,7 +15169,7 @@
     </row>
     <row r="1026" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1026" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B1026">
         <v>1907</v>
@@ -15183,7 +15183,7 @@
     </row>
     <row r="1027" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1027" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B1027">
         <v>1907</v>
@@ -15197,7 +15197,7 @@
     </row>
     <row r="1028" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1028" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B1028">
         <v>1907</v>
@@ -15211,7 +15211,7 @@
     </row>
     <row r="1029" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1029" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B1029">
         <v>1907</v>
@@ -15225,7 +15225,7 @@
     </row>
     <row r="1030" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1030" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B1030">
         <v>1907</v>
@@ -15239,7 +15239,7 @@
     </row>
     <row r="1031" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1031" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B1031">
         <v>1907</v>
@@ -15253,7 +15253,7 @@
     </row>
     <row r="1032" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1032" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B1032">
         <v>1907</v>
@@ -15267,7 +15267,7 @@
     </row>
     <row r="1033" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1033" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B1033">
         <v>1908</v>
@@ -15281,7 +15281,7 @@
     </row>
     <row r="1034" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1034" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B1034">
         <v>1908</v>
@@ -15295,7 +15295,7 @@
     </row>
     <row r="1035" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1035" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B1035">
         <v>1908</v>
@@ -15309,7 +15309,7 @@
     </row>
     <row r="1036" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1036" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B1036">
         <v>1908</v>
@@ -15323,7 +15323,7 @@
     </row>
     <row r="1037" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1037" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B1037">
         <v>1908</v>
@@ -15337,7 +15337,7 @@
     </row>
     <row r="1038" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1038" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B1038">
         <v>1908</v>
@@ -15351,7 +15351,7 @@
     </row>
     <row r="1039" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1039" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B1039">
         <v>1908</v>
@@ -15365,7 +15365,7 @@
     </row>
     <row r="1040" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1040" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B1040">
         <v>1908</v>
@@ -15379,7 +15379,7 @@
     </row>
     <row r="1041" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1041" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B1041">
         <v>1908</v>
@@ -15393,7 +15393,7 @@
     </row>
     <row r="1042" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1042" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1042">
         <v>2001</v>
@@ -15407,7 +15407,7 @@
     </row>
     <row r="1043" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1043" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1043">
         <v>2001</v>
@@ -15421,7 +15421,7 @@
     </row>
     <row r="1044" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1044" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1044">
         <v>2001</v>
@@ -15435,7 +15435,7 @@
     </row>
     <row r="1045" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1045" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1045">
         <v>2001</v>
@@ -15449,7 +15449,7 @@
     </row>
     <row r="1046" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1046" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1046">
         <v>2001</v>
@@ -15463,7 +15463,7 @@
     </row>
     <row r="1047" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1047" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1047">
         <v>2001</v>
@@ -15477,7 +15477,7 @@
     </row>
     <row r="1048" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1048" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1048">
         <v>2001</v>
@@ -15491,7 +15491,7 @@
     </row>
     <row r="1049" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1049" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1049">
         <v>2001</v>
@@ -15505,7 +15505,7 @@
     </row>
     <row r="1050" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1050" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1050">
         <v>2001</v>
@@ -15519,7 +15519,7 @@
     </row>
     <row r="1051" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1051" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1051">
         <v>2001</v>
@@ -15533,7 +15533,7 @@
     </row>
     <row r="1052" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1052" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1052">
         <v>2001</v>
@@ -15547,7 +15547,7 @@
     </row>
     <row r="1053" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1053" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1053">
         <v>2001</v>
@@ -15561,7 +15561,7 @@
     </row>
     <row r="1054" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1054" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1054">
         <v>2001</v>
@@ -15575,7 +15575,7 @@
     </row>
     <row r="1055" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1055" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1055">
         <v>2001</v>
@@ -15589,7 +15589,7 @@
     </row>
     <row r="1056" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1056" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1056">
         <v>2001</v>
@@ -15603,7 +15603,7 @@
     </row>
     <row r="1057" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1057" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1057">
         <v>2001</v>
@@ -15617,7 +15617,7 @@
     </row>
     <row r="1058" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1058" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1058">
         <v>2001</v>
@@ -15631,7 +15631,7 @@
     </row>
     <row r="1059" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1059" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1059">
         <v>2001</v>
@@ -15645,7 +15645,7 @@
     </row>
     <row r="1060" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1060" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1060">
         <v>2001</v>
@@ -15659,7 +15659,7 @@
     </row>
     <row r="1061" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1061" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1061">
         <v>2001</v>
@@ -15673,7 +15673,7 @@
     </row>
     <row r="1062" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1062" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1062">
         <v>2001</v>
@@ -15687,7 +15687,7 @@
     </row>
     <row r="1063" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1063" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B1063">
         <v>2001</v>
@@ -15701,7 +15701,7 @@
     </row>
     <row r="1064" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1064" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B1064">
         <v>2002</v>
@@ -15715,7 +15715,7 @@
     </row>
     <row r="1065" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1065" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B1065">
         <v>2002</v>
@@ -15729,7 +15729,7 @@
     </row>
     <row r="1066" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1066" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B1066">
         <v>2002</v>
@@ -15743,7 +15743,7 @@
     </row>
     <row r="1067" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1067" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B1067">
         <v>2002</v>
@@ -15757,7 +15757,7 @@
     </row>
     <row r="1068" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1068" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B1068">
         <v>2002</v>
@@ -15771,7 +15771,7 @@
     </row>
     <row r="1069" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1069" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B1069">
         <v>2002</v>
@@ -15785,7 +15785,7 @@
     </row>
     <row r="1070" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1070" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B1070">
         <v>2002</v>
@@ -15799,7 +15799,7 @@
     </row>
     <row r="1071" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1071" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B1071">
         <v>2002</v>
@@ -15813,7 +15813,7 @@
     </row>
     <row r="1072" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1072" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B1072">
         <v>2002</v>
@@ -15827,7 +15827,7 @@
     </row>
     <row r="1073" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1073" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B1073">
         <v>2002</v>
@@ -15841,7 +15841,7 @@
     </row>
     <row r="1074" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1074" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B1074">
         <v>2002</v>
@@ -15855,7 +15855,7 @@
     </row>
     <row r="1075" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1075" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B1075">
         <v>2002</v>
@@ -15869,7 +15869,7 @@
     </row>
     <row r="1076" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1076" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B1076">
         <v>2002</v>
@@ -15883,7 +15883,7 @@
     </row>
     <row r="1077" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1077" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B1077">
         <v>2002</v>
@@ -15897,7 +15897,7 @@
     </row>
     <row r="1078" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1078" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B1078">
         <v>2002</v>
@@ -15911,7 +15911,7 @@
     </row>
     <row r="1079" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1079" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B1079">
         <v>2002</v>
@@ -15925,7 +15925,7 @@
     </row>
     <row r="1080" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1080" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B1080">
         <v>2002</v>
@@ -15939,7 +15939,7 @@
     </row>
     <row r="1081" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1081" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B1081">
         <v>2002</v>
@@ -15953,7 +15953,7 @@
     </row>
     <row r="1082" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1082" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B1082">
         <v>2003</v>
@@ -15967,7 +15967,7 @@
     </row>
     <row r="1083" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1083" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B1083">
         <v>2003</v>
@@ -15981,7 +15981,7 @@
     </row>
     <row r="1084" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1084" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B1084">
         <v>2003</v>
@@ -15995,7 +15995,7 @@
     </row>
     <row r="1085" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1085" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B1085">
         <v>2003</v>
@@ -16009,7 +16009,7 @@
     </row>
     <row r="1086" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1086" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B1086">
         <v>2003</v>
@@ -16023,7 +16023,7 @@
     </row>
     <row r="1087" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1087" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B1087">
         <v>2003</v>
@@ -16037,7 +16037,7 @@
     </row>
     <row r="1088" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1088" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B1088">
         <v>2003</v>
@@ -16051,7 +16051,7 @@
     </row>
     <row r="1089" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1089" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B1089">
         <v>2003</v>
@@ -16065,7 +16065,7 @@
     </row>
     <row r="1090" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1090" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B1090">
         <v>2003</v>
@@ -16079,7 +16079,7 @@
     </row>
     <row r="1091" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1091" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B1091">
         <v>2003</v>
@@ -16093,7 +16093,7 @@
     </row>
     <row r="1092" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1092" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B1092">
         <v>2003</v>
@@ -16107,7 +16107,7 @@
     </row>
     <row r="1093" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1093" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B1093">
         <v>2003</v>
@@ -16121,7 +16121,7 @@
     </row>
     <row r="1094" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1094" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B1094">
         <v>2003</v>
@@ -16135,7 +16135,7 @@
     </row>
     <row r="1095" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1095" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B1095">
         <v>2003</v>
@@ -16149,7 +16149,7 @@
     </row>
     <row r="1096" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1096" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B1096">
         <v>2003</v>
@@ -16163,7 +16163,7 @@
     </row>
     <row r="1097" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1097" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B1097">
         <v>2003</v>
@@ -16177,7 +16177,7 @@
     </row>
     <row r="1098" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1098" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B1098">
         <v>2003</v>
@@ -16191,7 +16191,7 @@
     </row>
     <row r="1099" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1099" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B1099">
         <v>2003</v>
@@ -16205,7 +16205,7 @@
     </row>
     <row r="1100" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1100" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1100">
         <v>2101</v>
@@ -16219,7 +16219,7 @@
     </row>
     <row r="1101" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1101" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1101">
         <v>2101</v>
@@ -16233,7 +16233,7 @@
     </row>
     <row r="1102" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1102" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1102">
         <v>2101</v>
@@ -16247,7 +16247,7 @@
     </row>
     <row r="1103" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1103" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1103">
         <v>2101</v>
@@ -16261,7 +16261,7 @@
     </row>
     <row r="1104" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1104" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1104">
         <v>2101</v>
@@ -16275,7 +16275,7 @@
     </row>
     <row r="1105" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1105" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1105">
         <v>2101</v>
@@ -16289,7 +16289,7 @@
     </row>
     <row r="1106" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1106" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1106">
         <v>2101</v>
@@ -16303,7 +16303,7 @@
     </row>
     <row r="1107" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1107" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1107">
         <v>2101</v>
@@ -16317,7 +16317,7 @@
     </row>
     <row r="1108" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1108" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1108">
         <v>2101</v>
@@ -16331,7 +16331,7 @@
     </row>
     <row r="1109" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1109" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1109">
         <v>2101</v>
@@ -16345,7 +16345,7 @@
     </row>
     <row r="1110" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1110" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1110">
         <v>2101</v>
@@ -16359,7 +16359,7 @@
     </row>
     <row r="1111" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1111" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1111">
         <v>2101</v>
@@ -16373,7 +16373,7 @@
     </row>
     <row r="1112" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1112" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1112">
         <v>2101</v>
@@ -16387,7 +16387,7 @@
     </row>
     <row r="1113" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1113" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1113">
         <v>2101</v>
@@ -16401,7 +16401,7 @@
     </row>
     <row r="1114" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1114" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1114">
         <v>2101</v>
@@ -16415,7 +16415,7 @@
     </row>
     <row r="1115" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1115" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1115">
         <v>2101</v>
@@ -16429,7 +16429,7 @@
     </row>
     <row r="1116" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1116" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B1116">
         <v>2102</v>
@@ -16443,7 +16443,7 @@
     </row>
     <row r="1117" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1117" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B1117">
         <v>2102</v>
@@ -16457,7 +16457,7 @@
     </row>
     <row r="1118" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1118" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B1118">
         <v>2102</v>
@@ -16471,7 +16471,7 @@
     </row>
     <row r="1119" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1119" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B1119">
         <v>2102</v>
@@ -16485,7 +16485,7 @@
     </row>
     <row r="1120" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1120" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B1120">
         <v>2102</v>
@@ -16499,7 +16499,7 @@
     </row>
     <row r="1121" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1121" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B1121">
         <v>2102</v>
@@ -16513,7 +16513,7 @@
     </row>
     <row r="1122" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1122" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B1122">
         <v>2102</v>
@@ -16527,7 +16527,7 @@
     </row>
     <row r="1123" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1123" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B1123">
         <v>2102</v>
@@ -16541,7 +16541,7 @@
     </row>
     <row r="1124" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1124" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B1124">
         <v>2102</v>
@@ -16555,7 +16555,7 @@
     </row>
     <row r="1125" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1125" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B1125">
         <v>2102</v>
@@ -16569,7 +16569,7 @@
     </row>
     <row r="1126" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1126" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B1126">
         <v>2102</v>
@@ -16583,7 +16583,7 @@
     </row>
     <row r="1127" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1127" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B1127">
         <v>2102</v>
@@ -16597,7 +16597,7 @@
     </row>
     <row r="1128" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1128" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B1128">
         <v>2102</v>
@@ -16611,7 +16611,7 @@
     </row>
     <row r="1129" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1129" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1129">
         <v>2103</v>
@@ -16625,7 +16625,7 @@
     </row>
     <row r="1130" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1130" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1130">
         <v>2103</v>
@@ -16639,7 +16639,7 @@
     </row>
     <row r="1131" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1131" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1131">
         <v>2103</v>
@@ -16653,7 +16653,7 @@
     </row>
     <row r="1132" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1132" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1132">
         <v>2103</v>
@@ -16667,7 +16667,7 @@
     </row>
     <row r="1133" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1133" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1133">
         <v>2103</v>
@@ -16681,7 +16681,7 @@
     </row>
     <row r="1134" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1134" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1134">
         <v>2103</v>
@@ -16695,7 +16695,7 @@
     </row>
     <row r="1135" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1135" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1135">
         <v>2103</v>
@@ -16709,7 +16709,7 @@
     </row>
     <row r="1136" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1136" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1136">
         <v>2103</v>
@@ -16723,7 +16723,7 @@
     </row>
     <row r="1137" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1137" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1137">
         <v>2103</v>
@@ -16737,7 +16737,7 @@
     </row>
     <row r="1138" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1138" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1138">
         <v>2103</v>
@@ -16751,7 +16751,7 @@
     </row>
     <row r="1139" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1139" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1139">
         <v>2103</v>
@@ -16765,7 +16765,7 @@
     </row>
     <row r="1140" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1140" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1140">
         <v>2103</v>
@@ -16779,7 +16779,7 @@
     </row>
     <row r="1141" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1141" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1141">
         <v>2103</v>
@@ -16793,7 +16793,7 @@
     </row>
     <row r="1142" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1142" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1142">
         <v>2103</v>
@@ -16807,7 +16807,7 @@
     </row>
     <row r="1143" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1143" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1143">
         <v>2103</v>
@@ -16821,7 +16821,7 @@
     </row>
     <row r="1144" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1144" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1144">
         <v>2103</v>
@@ -16835,7 +16835,7 @@
     </row>
     <row r="1145" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1145" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1145">
         <v>2103</v>
@@ -16849,7 +16849,7 @@
     </row>
     <row r="1146" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1146" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1146">
         <v>2103</v>
@@ -16863,7 +16863,7 @@
     </row>
     <row r="1147" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1147" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1147">
         <v>2103</v>
@@ -16877,7 +16877,7 @@
     </row>
     <row r="1148" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1148" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1148">
         <v>2103</v>
@@ -16891,7 +16891,7 @@
     </row>
     <row r="1149" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1149" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1149">
         <v>2103</v>
@@ -16905,7 +16905,7 @@
     </row>
     <row r="1150" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1150" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1150">
         <v>2103</v>
@@ -16919,7 +16919,7 @@
     </row>
     <row r="1151" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1151" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1151">
         <v>2103</v>
@@ -16933,7 +16933,7 @@
     </row>
     <row r="1152" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1152" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1152">
         <v>2103</v>
@@ -16947,7 +16947,7 @@
     </row>
     <row r="1153" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1153" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1153">
         <v>2103</v>
@@ -16961,7 +16961,7 @@
     </row>
     <row r="1154" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1154" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1154">
         <v>2103</v>
@@ -16975,7 +16975,7 @@
     </row>
     <row r="1155" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1155" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1155">
         <v>2103</v>
@@ -16989,7 +16989,7 @@
     </row>
     <row r="1156" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1156" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1156">
         <v>2104</v>
@@ -17003,7 +17003,7 @@
     </row>
     <row r="1157" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1157" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1157">
         <v>2104</v>
@@ -17017,7 +17017,7 @@
     </row>
     <row r="1158" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1158" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1158">
         <v>2104</v>
@@ -17031,7 +17031,7 @@
     </row>
     <row r="1159" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1159" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1159">
         <v>2104</v>
@@ -17045,7 +17045,7 @@
     </row>
     <row r="1160" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1160" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1160">
         <v>2104</v>
@@ -17059,7 +17059,7 @@
     </row>
     <row r="1161" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1161" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1161">
         <v>2104</v>
@@ -17073,7 +17073,7 @@
     </row>
     <row r="1162" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1162" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1162">
         <v>2104</v>
@@ -17087,7 +17087,7 @@
     </row>
     <row r="1163" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1163" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1163">
         <v>2104</v>
@@ -17101,7 +17101,7 @@
     </row>
     <row r="1164" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1164" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1164">
         <v>2104</v>
@@ -17115,7 +17115,7 @@
     </row>
     <row r="1165" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1165" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1165">
         <v>2104</v>
@@ -17129,7 +17129,7 @@
     </row>
     <row r="1166" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1166" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1166">
         <v>2104</v>
@@ -17143,7 +17143,7 @@
     </row>
     <row r="1167" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1167" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1167">
         <v>2104</v>
@@ -17157,7 +17157,7 @@
     </row>
     <row r="1168" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1168" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1168">
         <v>2104</v>
@@ -17171,7 +17171,7 @@
     </row>
     <row r="1169" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1169" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1169">
         <v>2104</v>
@@ -17185,7 +17185,7 @@
     </row>
     <row r="1170" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1170" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1170">
         <v>2104</v>
@@ -17199,7 +17199,7 @@
     </row>
     <row r="1171" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1171" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1171">
         <v>2104</v>
@@ -17213,7 +17213,7 @@
     </row>
     <row r="1172" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1172" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1172">
         <v>2104</v>
@@ -17227,7 +17227,7 @@
     </row>
     <row r="1173" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1173" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1173">
         <v>2104</v>
@@ -17241,7 +17241,7 @@
     </row>
     <row r="1174" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1174" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1174">
         <v>2104</v>
@@ -17255,7 +17255,7 @@
     </row>
     <row r="1175" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1175" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1175">
         <v>2104</v>
@@ -17269,7 +17269,7 @@
     </row>
     <row r="1176" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1176" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1176">
         <v>2104</v>
@@ -17283,7 +17283,7 @@
     </row>
     <row r="1177" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1177" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1177">
         <v>2104</v>
@@ -17297,7 +17297,7 @@
     </row>
     <row r="1178" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1178" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1178">
         <v>2104</v>
@@ -17311,7 +17311,7 @@
     </row>
     <row r="1179" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1179" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1179">
         <v>2104</v>
@@ -17325,7 +17325,7 @@
     </row>
     <row r="1180" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1180" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B1180">
         <v>2105</v>
@@ -17339,7 +17339,7 @@
     </row>
     <row r="1181" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1181" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B1181">
         <v>2105</v>
@@ -17353,7 +17353,7 @@
     </row>
     <row r="1182" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1182" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B1182">
         <v>2105</v>
@@ -17367,7 +17367,7 @@
     </row>
     <row r="1183" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1183" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B1183">
         <v>2105</v>
@@ -17381,7 +17381,7 @@
     </row>
     <row r="1184" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1184" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B1184">
         <v>2105</v>
@@ -17395,7 +17395,7 @@
     </row>
     <row r="1185" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1185" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B1185">
         <v>2105</v>
@@ -17409,7 +17409,7 @@
     </row>
     <row r="1186" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1186" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B1186">
         <v>2105</v>
@@ -17423,7 +17423,7 @@
     </row>
     <row r="1187" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1187" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B1187">
         <v>2105</v>
@@ -17437,7 +17437,7 @@
     </row>
     <row r="1188" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1188" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B1188">
         <v>2105</v>
@@ -17451,7 +17451,7 @@
     </row>
     <row r="1189" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1189" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B1189">
         <v>2105</v>
@@ -17465,7 +17465,7 @@
     </row>
     <row r="1190" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1190" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B1190">
         <v>2105</v>
@@ -17479,7 +17479,7 @@
     </row>
     <row r="1191" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1191" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B1191">
         <v>2105</v>
@@ -17493,7 +17493,7 @@
     </row>
     <row r="1192" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1192" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B1192">
         <v>2105</v>
@@ -17507,7 +17507,7 @@
     </row>
     <row r="1193" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1193" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B1193">
         <v>2105</v>
@@ -17521,7 +17521,7 @@
     </row>
     <row r="1194" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1194" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B1194">
         <v>2105</v>
@@ -17535,7 +17535,7 @@
     </row>
     <row r="1195" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1195" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B1195">
         <v>2105</v>
@@ -17549,7 +17549,7 @@
     </row>
     <row r="1196" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1196" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B1196">
         <v>2105</v>
@@ -17563,7 +17563,7 @@
     </row>
     <row r="1197" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1197" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B1197">
         <v>2105</v>
@@ -17577,7 +17577,7 @@
     </row>
     <row r="1198" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1198" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B1198">
         <v>2105</v>
@@ -17591,7 +17591,7 @@
     </row>
     <row r="1199" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1199" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B1199">
         <v>2106</v>
@@ -17605,7 +17605,7 @@
     </row>
     <row r="1200" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1200" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B1200">
         <v>2106</v>
@@ -17619,7 +17619,7 @@
     </row>
     <row r="1201" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1201" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B1201">
         <v>2106</v>
@@ -17633,7 +17633,7 @@
     </row>
     <row r="1202" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1202" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B1202">
         <v>2106</v>
@@ -17647,7 +17647,7 @@
     </row>
     <row r="1203" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1203" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B1203">
         <v>2106</v>
@@ -17661,7 +17661,7 @@
     </row>
     <row r="1204" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1204" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B1204">
         <v>2106</v>
@@ -17675,7 +17675,7 @@
     </row>
     <row r="1205" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1205" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B1205">
         <v>2106</v>
@@ -17689,7 +17689,7 @@
     </row>
     <row r="1206" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1206" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B1206">
         <v>2106</v>
@@ -17703,7 +17703,7 @@
     </row>
     <row r="1207" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1207" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B1207">
         <v>2106</v>
@@ -17717,7 +17717,7 @@
     </row>
     <row r="1208" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1208" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B1208">
         <v>2106</v>
@@ -17731,7 +17731,7 @@
     </row>
     <row r="1209" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1209" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B1209">
         <v>2106</v>
@@ -17745,7 +17745,7 @@
     </row>
     <row r="1210" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1210" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B1210">
         <v>2106</v>
@@ -17759,7 +17759,7 @@
     </row>
     <row r="1211" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1211" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B1211">
         <v>2106</v>
@@ -17773,7 +17773,7 @@
     </row>
     <row r="1212" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1212" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B1212">
         <v>2106</v>
@@ -17787,7 +17787,7 @@
     </row>
     <row r="1213" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1213" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B1213">
         <v>2107</v>
@@ -17801,7 +17801,7 @@
     </row>
     <row r="1214" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1214" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B1214">
         <v>2107</v>
@@ -17815,7 +17815,7 @@
     </row>
     <row r="1215" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1215" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B1215">
         <v>2107</v>
@@ -17829,7 +17829,7 @@
     </row>
     <row r="1216" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1216" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B1216">
         <v>2107</v>
@@ -17843,7 +17843,7 @@
     </row>
     <row r="1217" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1217" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B1217">
         <v>2107</v>
@@ -17857,7 +17857,7 @@
     </row>
     <row r="1218" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1218" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B1218">
         <v>2107</v>
@@ -17871,7 +17871,7 @@
     </row>
     <row r="1219" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1219" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B1219">
         <v>2107</v>
@@ -17885,7 +17885,7 @@
     </row>
     <row r="1220" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1220" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B1220">
         <v>2107</v>
@@ -17899,7 +17899,7 @@
     </row>
     <row r="1221" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1221" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B1221">
         <v>2107</v>
@@ -17913,7 +17913,7 @@
     </row>
     <row r="1222" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1222" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B1222">
         <v>2107</v>
@@ -17927,7 +17927,7 @@
     </row>
     <row r="1223" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1223" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B1223">
         <v>2108</v>
@@ -17941,7 +17941,7 @@
     </row>
     <row r="1224" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1224" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B1224">
         <v>2108</v>
@@ -17955,7 +17955,7 @@
     </row>
     <row r="1225" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1225" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B1225">
         <v>2108</v>
@@ -17969,7 +17969,7 @@
     </row>
     <row r="1226" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1226" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B1226">
         <v>2108</v>
@@ -17983,7 +17983,7 @@
     </row>
     <row r="1227" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1227" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B1227">
         <v>2108</v>
@@ -17997,7 +17997,7 @@
     </row>
     <row r="1228" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1228" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B1228">
         <v>2108</v>
@@ -18011,7 +18011,7 @@
     </row>
     <row r="1229" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1229" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B1229">
         <v>2108</v>
@@ -18025,7 +18025,7 @@
     </row>
     <row r="1230" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1230" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B1230">
         <v>2109</v>
@@ -18039,7 +18039,7 @@
     </row>
     <row r="1231" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1231" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B1231">
         <v>2109</v>
@@ -18053,7 +18053,7 @@
     </row>
     <row r="1232" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1232" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B1232">
         <v>2109</v>
@@ -18067,7 +18067,7 @@
     </row>
     <row r="1233" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1233" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B1233">
         <v>2109</v>
@@ -18081,7 +18081,7 @@
     </row>
     <row r="1234" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1234" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B1234">
         <v>2201</v>
@@ -18095,7 +18095,7 @@
     </row>
     <row r="1235" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1235" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B1235">
         <v>2201</v>
@@ -18109,7 +18109,7 @@
     </row>
     <row r="1236" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1236" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B1236">
         <v>2201</v>
@@ -18123,7 +18123,7 @@
     </row>
     <row r="1237" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1237" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B1237">
         <v>2201</v>
@@ -18137,7 +18137,7 @@
     </row>
     <row r="1238" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1238" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B1238">
         <v>2201</v>
@@ -18151,7 +18151,7 @@
     </row>
     <row r="1239" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1239" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B1239">
         <v>2201</v>
@@ -18165,7 +18165,7 @@
     </row>
     <row r="1240" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1240" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B1240">
         <v>2202</v>
@@ -18179,7 +18179,7 @@
     </row>
     <row r="1241" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1241" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B1241">
         <v>2202</v>
@@ -18193,7 +18193,7 @@
     </row>
     <row r="1242" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1242" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B1242">
         <v>2202</v>
@@ -18207,7 +18207,7 @@
     </row>
     <row r="1243" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1243" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B1243">
         <v>2202</v>
@@ -18221,7 +18221,7 @@
     </row>
     <row r="1244" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1244" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B1244">
         <v>2202</v>
@@ -18235,7 +18235,7 @@
     </row>
     <row r="1245" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1245" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B1245">
         <v>2202</v>
@@ -18249,7 +18249,7 @@
     </row>
     <row r="1246" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1246" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B1246">
         <v>2202</v>
@@ -18263,7 +18263,7 @@
     </row>
     <row r="1247" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1247" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B1247">
         <v>2202</v>
@@ -18277,7 +18277,7 @@
     </row>
     <row r="1248" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1248" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B1248">
         <v>2202</v>
@@ -18291,7 +18291,7 @@
     </row>
     <row r="1249" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1249" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B1249">
         <v>2202</v>
@@ -18305,7 +18305,7 @@
     </row>
     <row r="1250" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1250" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B1250">
         <v>2202</v>
@@ -18319,7 +18319,7 @@
     </row>
     <row r="1251" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1251" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B1251">
         <v>2202</v>
@@ -18333,7 +18333,7 @@
     </row>
     <row r="1252" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1252" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B1252">
         <v>2202</v>
@@ -18347,7 +18347,7 @@
     </row>
     <row r="1253" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1253" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B1253">
         <v>2202</v>
@@ -18361,7 +18361,7 @@
     </row>
     <row r="1254" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1254" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B1254">
         <v>2202</v>
@@ -18375,7 +18375,7 @@
     </row>
     <row r="1255" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1255" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B1255">
         <v>2202</v>
@@ -18389,7 +18389,7 @@
     </row>
     <row r="1256" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1256" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B1256">
         <v>2203</v>
@@ -18403,7 +18403,7 @@
     </row>
     <row r="1257" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1257" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B1257">
         <v>2203</v>
@@ -18417,7 +18417,7 @@
     </row>
     <row r="1258" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1258" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B1258">
         <v>2203</v>
@@ -18431,7 +18431,7 @@
     </row>
     <row r="1259" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1259" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B1259">
         <v>2203</v>
@@ -18445,7 +18445,7 @@
     </row>
     <row r="1260" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1260" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B1260">
         <v>2203</v>
@@ -18459,7 +18459,7 @@
     </row>
     <row r="1261" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1261" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B1261">
         <v>2203</v>
@@ -18473,7 +18473,7 @@
     </row>
     <row r="1262" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1262" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B1262">
         <v>2203</v>
@@ -18487,7 +18487,7 @@
     </row>
     <row r="1263" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1263" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B1263">
         <v>2203</v>
@@ -18501,7 +18501,7 @@
     </row>
     <row r="1264" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1264" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B1264">
         <v>2203</v>
@@ -18515,7 +18515,7 @@
     </row>
     <row r="1265" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1265" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B1265">
         <v>2203</v>
@@ -18529,7 +18529,7 @@
     </row>
     <row r="1266" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1266" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B1266">
         <v>2203</v>
@@ -18543,7 +18543,7 @@
     </row>
     <row r="1267" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1267" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B1267">
         <v>2203</v>
@@ -18557,7 +18557,7 @@
     </row>
     <row r="1268" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1268" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B1268">
         <v>2203</v>
@@ -18571,7 +18571,7 @@
     </row>
     <row r="1269" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1269" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B1269">
         <v>2204</v>
@@ -18585,7 +18585,7 @@
     </row>
     <row r="1270" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1270" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B1270">
         <v>2204</v>
@@ -18599,7 +18599,7 @@
     </row>
     <row r="1271" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1271" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B1271">
         <v>2204</v>
@@ -18613,7 +18613,7 @@
     </row>
     <row r="1272" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1272" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B1272">
         <v>2204</v>
@@ -18627,7 +18627,7 @@
     </row>
     <row r="1273" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1273" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B1273">
         <v>2205</v>
@@ -18641,7 +18641,7 @@
     </row>
     <row r="1274" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1274" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B1274">
         <v>2205</v>
@@ -18655,7 +18655,7 @@
     </row>
     <row r="1275" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1275" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B1275">
         <v>2205</v>
@@ -18669,7 +18669,7 @@
     </row>
     <row r="1276" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1276" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B1276">
         <v>2205</v>
@@ -18683,7 +18683,7 @@
     </row>
     <row r="1277" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1277" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B1277">
         <v>2205</v>
@@ -18697,7 +18697,7 @@
     </row>
     <row r="1278" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1278" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B1278">
         <v>2205</v>
@@ -18711,7 +18711,7 @@
     </row>
     <row r="1279" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1279" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B1279">
         <v>2205</v>
@@ -18725,7 +18725,7 @@
     </row>
     <row r="1280" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1280" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B1280">
         <v>2205</v>
@@ -18739,7 +18739,7 @@
     </row>
     <row r="1281" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1281" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B1281">
         <v>2205</v>
@@ -18753,7 +18753,7 @@
     </row>
     <row r="1282" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1282" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B1282">
         <v>2205</v>
@@ -18767,7 +18767,7 @@
     </row>
     <row r="1283" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1283" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B1283">
         <v>2205</v>
@@ -18781,7 +18781,7 @@
     </row>
     <row r="1284" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1284" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B1284">
         <v>2205</v>
@@ -18795,7 +18795,7 @@
     </row>
     <row r="1285" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1285" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B1285">
         <v>2205</v>
@@ -18809,7 +18809,7 @@
     </row>
     <row r="1286" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1286" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B1286">
         <v>2205</v>
@@ -18823,7 +18823,7 @@
     </row>
     <row r="1287" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1287" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B1287">
         <v>2205</v>
@@ -18837,7 +18837,7 @@
     </row>
     <row r="1288" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1288" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B1288">
         <v>2205</v>
@@ -18851,7 +18851,7 @@
     </row>
     <row r="1289" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1289" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B1289">
         <v>2206</v>
@@ -18865,7 +18865,7 @@
     </row>
     <row r="1290" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1290" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B1290">
         <v>2206</v>
@@ -18879,7 +18879,7 @@
     </row>
     <row r="1291" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1291" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B1291">
         <v>2206</v>
@@ -18893,7 +18893,7 @@
     </row>
     <row r="1292" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1292" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B1292">
         <v>2206</v>
@@ -18907,7 +18907,7 @@
     </row>
     <row r="1293" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1293" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B1293">
         <v>2206</v>
@@ -18921,7 +18921,7 @@
     </row>
     <row r="1294" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1294" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B1294">
         <v>2206</v>
@@ -18935,7 +18935,7 @@
     </row>
     <row r="1295" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1295" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B1295">
         <v>2206</v>
@@ -18949,7 +18949,7 @@
     </row>
     <row r="1296" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1296" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B1296">
         <v>2206</v>
@@ -18963,7 +18963,7 @@
     </row>
     <row r="1297" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1297" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B1297">
         <v>2206</v>
@@ -18977,7 +18977,7 @@
     </row>
     <row r="1298" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1298" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B1298">
         <v>2206</v>
@@ -18991,7 +18991,7 @@
     </row>
     <row r="1299" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1299" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B1299">
         <v>2206</v>
@@ -19005,7 +19005,7 @@
     </row>
     <row r="1300" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1300" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B1300">
         <v>2206</v>
@@ -19019,7 +19019,7 @@
     </row>
     <row r="1301" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1301" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B1301">
         <v>2206</v>
@@ -19033,7 +19033,7 @@
     </row>
     <row r="1302" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1302" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B1302">
         <v>2206</v>
@@ -19047,7 +19047,7 @@
     </row>
     <row r="1303" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1303" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B1303">
         <v>2206</v>
@@ -19061,7 +19061,7 @@
     </row>
     <row r="1304" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1304" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B1304">
         <v>2206</v>
@@ -19075,7 +19075,7 @@
     </row>
     <row r="1305" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1305" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1305">
         <v>2207</v>
@@ -19089,7 +19089,7 @@
     </row>
     <row r="1306" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1306" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1306">
         <v>2207</v>
@@ -19103,7 +19103,7 @@
     </row>
     <row r="1307" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1307" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1307">
         <v>2207</v>
@@ -19117,7 +19117,7 @@
     </row>
     <row r="1308" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1308" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1308">
         <v>2207</v>
@@ -19131,7 +19131,7 @@
     </row>
     <row r="1309" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1309" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1309">
         <v>2207</v>
@@ -19145,7 +19145,7 @@
     </row>
     <row r="1310" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1310" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1310">
         <v>2207</v>
@@ -19159,7 +19159,7 @@
     </row>
     <row r="1311" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1311" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1311">
         <v>2207</v>
@@ -19173,7 +19173,7 @@
     </row>
     <row r="1312" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1312" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1312">
         <v>2207</v>
@@ -19187,7 +19187,7 @@
     </row>
     <row r="1313" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1313" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1313">
         <v>2207</v>
@@ -19201,7 +19201,7 @@
     </row>
     <row r="1314" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1314" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1314">
         <v>2207</v>
@@ -19215,7 +19215,7 @@
     </row>
     <row r="1315" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1315" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1315">
         <v>2207</v>
@@ -19229,7 +19229,7 @@
     </row>
     <row r="1316" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1316" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1316">
         <v>2207</v>
@@ -19243,7 +19243,7 @@
     </row>
     <row r="1317" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1317" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1317">
         <v>2207</v>
@@ -19257,7 +19257,7 @@
     </row>
     <row r="1318" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1318" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1318">
         <v>2207</v>
@@ -19271,7 +19271,7 @@
     </row>
     <row r="1319" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1319" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1319">
         <v>2207</v>
@@ -19285,7 +19285,7 @@
     </row>
     <row r="1320" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1320" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1320">
         <v>2207</v>
@@ -19299,7 +19299,7 @@
     </row>
     <row r="1321" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1321" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1321">
         <v>2207</v>
@@ -19313,7 +19313,7 @@
     </row>
     <row r="1322" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1322" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1322">
         <v>2207</v>
@@ -19327,7 +19327,7 @@
     </row>
     <row r="1323" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1323" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1323">
         <v>2207</v>
@@ -19341,7 +19341,7 @@
     </row>
     <row r="1324" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1324" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1324">
         <v>2207</v>
@@ -19355,7 +19355,7 @@
     </row>
     <row r="1325" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1325" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1325">
         <v>2207</v>
@@ -19369,7 +19369,7 @@
     </row>
     <row r="1326" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1326" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1326">
         <v>2207</v>
@@ -19383,7 +19383,7 @@
     </row>
     <row r="1327" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1327" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1327">
         <v>2207</v>
@@ -19397,7 +19397,7 @@
     </row>
     <row r="1328" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1328" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1328">
         <v>2207</v>
@@ -19411,7 +19411,7 @@
     </row>
     <row r="1329" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1329" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1329">
         <v>2207</v>
@@ -19425,7 +19425,7 @@
     </row>
     <row r="1330" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1330" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1330">
         <v>2207</v>
@@ -19439,7 +19439,7 @@
     </row>
     <row r="1331" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1331" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1331">
         <v>2207</v>
@@ -19453,7 +19453,7 @@
     </row>
     <row r="1332" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1332" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1332">
         <v>2207</v>
@@ -19467,7 +19467,7 @@
     </row>
     <row r="1333" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1333" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1333">
         <v>2207</v>
@@ -19481,7 +19481,7 @@
     </row>
     <row r="1334" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1334" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1334">
         <v>2207</v>
@@ -19495,7 +19495,7 @@
     </row>
     <row r="1335" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1335" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1335">
         <v>2207</v>
@@ -19509,7 +19509,7 @@
     </row>
     <row r="1336" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1336" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B1336">
         <v>2207</v>
@@ -19523,7 +19523,7 @@
     </row>
     <row r="1337" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1337" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B1337">
         <v>2208</v>
@@ -19537,7 +19537,7 @@
     </row>
     <row r="1338" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1338" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B1338">
         <v>2208</v>
@@ -19551,7 +19551,7 @@
     </row>
     <row r="1339" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1339" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B1339">
         <v>2208</v>
@@ -19565,7 +19565,7 @@
     </row>
     <row r="1340" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1340" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B1340">
         <v>2208</v>
@@ -19579,7 +19579,7 @@
     </row>
     <row r="1341" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1341" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B1341">
         <v>2208</v>
@@ -19593,7 +19593,7 @@
     </row>
     <row r="1342" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1342" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B1342">
         <v>2208</v>
@@ -19607,7 +19607,7 @@
     </row>
     <row r="1343" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1343" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B1343">
         <v>2208</v>
@@ -19621,7 +19621,7 @@
     </row>
     <row r="1344" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1344" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B1344">
         <v>2208</v>
@@ -19635,7 +19635,7 @@
     </row>
     <row r="1345" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1345" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B1345">
         <v>2208</v>
@@ -19649,7 +19649,7 @@
     </row>
     <row r="1346" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1346" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B1346">
         <v>2210</v>
@@ -19663,7 +19663,7 @@
     </row>
     <row r="1347" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1347" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B1347">
         <v>2210</v>
@@ -19677,7 +19677,7 @@
     </row>
     <row r="1348" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1348" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B1348">
         <v>2210</v>
@@ -19691,7 +19691,7 @@
     </row>
     <row r="1349" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1349" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B1349">
         <v>2210</v>
@@ -19705,7 +19705,7 @@
     </row>
     <row r="1350" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1350" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B1350">
         <v>2210</v>
@@ -19719,7 +19719,7 @@
     </row>
     <row r="1351" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1351" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B1351">
         <v>2210</v>
@@ -19733,7 +19733,7 @@
     </row>
     <row r="1352" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1352" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B1352">
         <v>2210</v>
@@ -19747,7 +19747,7 @@
     </row>
     <row r="1353" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1353" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B1353">
         <v>2210</v>
@@ -19761,7 +19761,7 @@
     </row>
     <row r="1354" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1354" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B1354">
         <v>2210</v>
@@ -19775,7 +19775,7 @@
     </row>
     <row r="1355" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1355" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B1355">
         <v>2210</v>
@@ -19789,7 +19789,7 @@
     </row>
     <row r="1356" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1356" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B1356">
         <v>2210</v>
@@ -19803,7 +19803,7 @@
     </row>
     <row r="1357" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1357" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B1357">
         <v>2210</v>
@@ -19817,7 +19817,7 @@
     </row>
     <row r="1358" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1358" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B1358">
         <v>2210</v>
@@ -19831,7 +19831,7 @@
     </row>
     <row r="1359" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1359" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B1359">
         <v>2210</v>
@@ -19845,7 +19845,7 @@
     </row>
     <row r="1360" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1360" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B1360">
         <v>2211</v>
@@ -19859,7 +19859,7 @@
     </row>
     <row r="1361" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1361" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B1361">
         <v>2211</v>
@@ -19873,7 +19873,7 @@
     </row>
     <row r="1362" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1362" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B1362">
         <v>2211</v>
@@ -19887,7 +19887,7 @@
     </row>
     <row r="1363" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1363" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B1363">
         <v>2211</v>
@@ -19901,7 +19901,7 @@
     </row>
     <row r="1364" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1364" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B1364">
         <v>2211</v>
@@ -19915,7 +19915,7 @@
     </row>
     <row r="1365" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1365" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B1365">
         <v>2211</v>
@@ -19929,7 +19929,7 @@
     </row>
     <row r="1366" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1366" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B1366">
         <v>2211</v>
@@ -19943,7 +19943,7 @@
     </row>
     <row r="1367" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1367" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B1367">
         <v>2212</v>
@@ -19957,7 +19957,7 @@
     </row>
     <row r="1368" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1368" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B1368">
         <v>2212</v>
@@ -19971,7 +19971,7 @@
     </row>
     <row r="1369" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1369" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B1369">
         <v>2212</v>
@@ -19985,7 +19985,7 @@
     </row>
     <row r="1370" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1370" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B1370">
         <v>2212</v>
@@ -19999,7 +19999,7 @@
     </row>
     <row r="1371" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1371" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B1371">
         <v>2212</v>
@@ -20013,7 +20013,7 @@
     </row>
     <row r="1372" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1372" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B1372">
         <v>2212</v>
@@ -20027,7 +20027,7 @@
     </row>
     <row r="1373" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1373" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B1373">
         <v>2212</v>
@@ -20041,7 +20041,7 @@
     </row>
     <row r="1374" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1374" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1374">
         <v>2213</v>
@@ -20055,7 +20055,7 @@
     </row>
     <row r="1375" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1375" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1375">
         <v>2213</v>
@@ -20069,7 +20069,7 @@
     </row>
     <row r="1376" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1376" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1376">
         <v>2213</v>
@@ -20083,7 +20083,7 @@
     </row>
     <row r="1377" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1377" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1377">
         <v>2213</v>
@@ -20097,7 +20097,7 @@
     </row>
     <row r="1378" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1378" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1378">
         <v>2213</v>
@@ -20111,7 +20111,7 @@
     </row>
     <row r="1379" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1379" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1379">
         <v>2213</v>
@@ -20125,7 +20125,7 @@
     </row>
     <row r="1380" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1380" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1380">
         <v>2213</v>
@@ -20139,7 +20139,7 @@
     </row>
     <row r="1381" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1381" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1381">
         <v>2213</v>
@@ -20153,7 +20153,7 @@
     </row>
     <row r="1382" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1382" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1382">
         <v>2213</v>
@@ -20167,7 +20167,7 @@
     </row>
     <row r="1383" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1383" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1383">
         <v>2213</v>
@@ -20181,7 +20181,7 @@
     </row>
     <row r="1384" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1384" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1384">
         <v>2213</v>
@@ -20195,7 +20195,7 @@
     </row>
     <row r="1385" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1385" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1385">
         <v>2213</v>
@@ -20209,7 +20209,7 @@
     </row>
     <row r="1386" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1386" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1386">
         <v>2213</v>
@@ -20223,7 +20223,7 @@
     </row>
     <row r="1387" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1387" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1387">
         <v>2213</v>
@@ -20237,7 +20237,7 @@
     </row>
     <row r="1388" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1388" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1388">
         <v>2213</v>
@@ -20251,7 +20251,7 @@
     </row>
     <row r="1389" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1389" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1389">
         <v>2213</v>
@@ -20265,7 +20265,7 @@
     </row>
     <row r="1390" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1390" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1390">
         <v>2213</v>
@@ -20279,7 +20279,7 @@
     </row>
     <row r="1391" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1391" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1391">
         <v>2213</v>
@@ -20293,7 +20293,7 @@
     </row>
     <row r="1392" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1392" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1392">
         <v>2213</v>
@@ -20307,7 +20307,7 @@
     </row>
     <row r="1393" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1393" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1393">
         <v>2213</v>
@@ -20321,7 +20321,7 @@
     </row>
     <row r="1394" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1394" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1394">
         <v>2213</v>
@@ -20335,7 +20335,7 @@
     </row>
     <row r="1395" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1395" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1395">
         <v>2213</v>
@@ -20349,7 +20349,7 @@
     </row>
     <row r="1396" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1396" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1396">
         <v>2213</v>
@@ -20363,7 +20363,7 @@
     </row>
     <row r="1397" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1397" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B1397">
         <v>2213</v>
@@ -20377,7 +20377,7 @@
     </row>
     <row r="1398" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1398" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B1398">
         <v>2215</v>
@@ -20391,7 +20391,7 @@
     </row>
     <row r="1399" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1399" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B1399">
         <v>2215</v>
@@ -20405,7 +20405,7 @@
     </row>
     <row r="1400" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1400" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B1400">
         <v>2215</v>
@@ -20419,7 +20419,7 @@
     </row>
     <row r="1401" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1401" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B1401">
         <v>2215</v>
@@ -20433,7 +20433,7 @@
     </row>
     <row r="1402" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1402" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B1402">
         <v>2215</v>
@@ -20447,7 +20447,7 @@
     </row>
     <row r="1403" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1403" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1403">
         <v>2301</v>
@@ -20461,7 +20461,7 @@
     </row>
     <row r="1404" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1404" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1404">
         <v>2301</v>
@@ -20475,7 +20475,7 @@
     </row>
     <row r="1405" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1405" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1405">
         <v>2301</v>
@@ -20489,7 +20489,7 @@
     </row>
     <row r="1406" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1406" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1406">
         <v>2301</v>
@@ -20503,7 +20503,7 @@
     </row>
     <row r="1407" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1407" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1407">
         <v>2301</v>
@@ -20517,7 +20517,7 @@
     </row>
     <row r="1408" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1408" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1408">
         <v>2301</v>
@@ -20531,7 +20531,7 @@
     </row>
     <row r="1409" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1409" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1409">
         <v>2301</v>
@@ -20545,7 +20545,7 @@
     </row>
     <row r="1410" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1410" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1410">
         <v>2301</v>
@@ -20559,7 +20559,7 @@
     </row>
     <row r="1411" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1411" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1411">
         <v>2301</v>
@@ -20573,7 +20573,7 @@
     </row>
     <row r="1412" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1412" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1412">
         <v>2301</v>
@@ -20587,7 +20587,7 @@
     </row>
     <row r="1413" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1413" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1413">
         <v>2301</v>
@@ -20601,7 +20601,7 @@
     </row>
     <row r="1414" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1414" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1414">
         <v>2301</v>
@@ -20615,7 +20615,7 @@
     </row>
     <row r="1415" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1415" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1415">
         <v>2301</v>
@@ -20629,7 +20629,7 @@
     </row>
     <row r="1416" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1416" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1416">
         <v>2301</v>
@@ -20643,7 +20643,7 @@
     </row>
     <row r="1417" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1417" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1417">
         <v>2301</v>
@@ -20657,7 +20657,7 @@
     </row>
     <row r="1418" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1418" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1418">
         <v>2301</v>
@@ -20671,7 +20671,7 @@
     </row>
     <row r="1419" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1419" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1419">
         <v>2301</v>
@@ -20685,7 +20685,7 @@
     </row>
     <row r="1420" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1420" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1420">
         <v>2301</v>
@@ -20699,7 +20699,7 @@
     </row>
     <row r="1421" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1421" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1421">
         <v>2301</v>
@@ -20713,7 +20713,7 @@
     </row>
     <row r="1422" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1422" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1422">
         <v>2301</v>
@@ -20727,7 +20727,7 @@
     </row>
     <row r="1423" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1423" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1423">
         <v>2301</v>
@@ -20741,7 +20741,7 @@
     </row>
     <row r="1424" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1424" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1424">
         <v>2301</v>
@@ -20755,7 +20755,7 @@
     </row>
     <row r="1425" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1425" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1425">
         <v>2301</v>
@@ -20769,7 +20769,7 @@
     </row>
     <row r="1426" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1426" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1426">
         <v>2301</v>
@@ -20783,7 +20783,7 @@
     </row>
     <row r="1427" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1427" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1427">
         <v>2301</v>
@@ -20797,7 +20797,7 @@
     </row>
     <row r="1428" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1428" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1428">
         <v>2301</v>
@@ -20811,7 +20811,7 @@
     </row>
     <row r="1429" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1429" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1429">
         <v>2301</v>
@@ -20825,7 +20825,7 @@
     </row>
     <row r="1430" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1430" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1430">
         <v>2302</v>
@@ -20839,7 +20839,7 @@
     </row>
     <row r="1431" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1431" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1431">
         <v>2302</v>
@@ -20853,7 +20853,7 @@
     </row>
     <row r="1432" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1432" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1432">
         <v>2302</v>
@@ -20867,7 +20867,7 @@
     </row>
     <row r="1433" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1433" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1433">
         <v>2302</v>
@@ -20881,7 +20881,7 @@
     </row>
     <row r="1434" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1434" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1434">
         <v>2302</v>
@@ -20895,7 +20895,7 @@
     </row>
     <row r="1435" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1435" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1435">
         <v>2302</v>
@@ -20909,7 +20909,7 @@
     </row>
     <row r="1436" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1436" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1436">
         <v>2302</v>
@@ -20923,7 +20923,7 @@
     </row>
     <row r="1437" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1437" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1437">
         <v>2302</v>
@@ -20937,7 +20937,7 @@
     </row>
     <row r="1438" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1438" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1438">
         <v>2302</v>
@@ -20951,7 +20951,7 @@
     </row>
     <row r="1439" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1439" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1439">
         <v>2302</v>
@@ -20965,7 +20965,7 @@
     </row>
     <row r="1440" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1440" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1440">
         <v>2302</v>
@@ -20979,7 +20979,7 @@
     </row>
     <row r="1441" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1441" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1441">
         <v>2302</v>
@@ -20993,7 +20993,7 @@
     </row>
     <row r="1442" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1442" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1442">
         <v>2302</v>
@@ -21007,7 +21007,7 @@
     </row>
     <row r="1443" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1443" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1443">
         <v>2302</v>
@@ -21021,7 +21021,7 @@
     </row>
     <row r="1444" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1444" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1444">
         <v>2302</v>
@@ -21035,7 +21035,7 @@
     </row>
     <row r="1445" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1445" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1445">
         <v>2302</v>
@@ -21049,7 +21049,7 @@
     </row>
     <row r="1446" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1446" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1446">
         <v>2302</v>
@@ -21063,7 +21063,7 @@
     </row>
     <row r="1447" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1447" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1447">
         <v>2302</v>
@@ -21077,7 +21077,7 @@
     </row>
     <row r="1448" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1448" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B1448">
         <v>2302</v>
@@ -21091,7 +21091,7 @@
     </row>
     <row r="1449" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1449" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1449">
         <v>2303</v>
@@ -21105,7 +21105,7 @@
     </row>
     <row r="1450" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1450" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1450">
         <v>2303</v>
@@ -21119,7 +21119,7 @@
     </row>
     <row r="1451" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1451" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1451">
         <v>2303</v>
@@ -21133,7 +21133,7 @@
     </row>
     <row r="1452" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1452" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1452">
         <v>2303</v>
@@ -21147,7 +21147,7 @@
     </row>
     <row r="1453" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1453" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1453">
         <v>2303</v>
@@ -21161,7 +21161,7 @@
     </row>
     <row r="1454" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1454" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1454">
         <v>2303</v>
@@ -21175,7 +21175,7 @@
     </row>
     <row r="1455" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1455" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1455">
         <v>2303</v>
@@ -21189,7 +21189,7 @@
     </row>
     <row r="1456" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1456" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1456">
         <v>2303</v>
@@ -21203,7 +21203,7 @@
     </row>
     <row r="1457" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1457" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1457">
         <v>2303</v>
@@ -21217,7 +21217,7 @@
     </row>
     <row r="1458" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1458" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1458">
         <v>2303</v>
@@ -21231,7 +21231,7 @@
     </row>
     <row r="1459" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1459" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1459">
         <v>2303</v>
@@ -21245,7 +21245,7 @@
     </row>
     <row r="1460" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1460" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1460">
         <v>2303</v>
@@ -21259,7 +21259,7 @@
     </row>
     <row r="1461" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1461" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1461">
         <v>2303</v>
@@ -21273,7 +21273,7 @@
     </row>
     <row r="1462" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1462" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B1462">
         <v>2303</v>
@@ -21287,7 +21287,7 @@
     </row>
     <row r="1463" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1463" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B1463">
         <v>2304</v>
@@ -21301,7 +21301,7 @@
     </row>
     <row r="1464" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1464" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B1464">
         <v>2304</v>
@@ -21315,7 +21315,7 @@
     </row>
     <row r="1465" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1465" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B1465">
         <v>2304</v>
@@ -21329,7 +21329,7 @@
     </row>
     <row r="1466" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1466" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B1466">
         <v>2304</v>
@@ -21343,7 +21343,7 @@
     </row>
     <row r="1467" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1467" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B1467">
         <v>2304</v>
@@ -21357,7 +21357,7 @@
     </row>
     <row r="1468" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1468" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B1468">
         <v>2304</v>
@@ -21371,7 +21371,7 @@
     </row>
     <row r="1469" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1469" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B1469">
         <v>2304</v>
@@ -21385,7 +21385,7 @@
     </row>
     <row r="1470" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1470" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B1470">
         <v>2304</v>
@@ -21399,7 +21399,7 @@
     </row>
     <row r="1471" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1471" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B1471">
         <v>2304</v>
@@ -21413,7 +21413,7 @@
     </row>
     <row r="1472" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1472" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B1472">
         <v>2305</v>
@@ -21427,7 +21427,7 @@
     </row>
     <row r="1473" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1473" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B1473">
         <v>2305</v>
@@ -21441,7 +21441,7 @@
     </row>
     <row r="1474" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1474" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B1474">
         <v>2305</v>
@@ -21455,7 +21455,7 @@
     </row>
     <row r="1475" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1475" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B1475">
         <v>2305</v>
@@ -21469,7 +21469,7 @@
     </row>
     <row r="1476" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1476" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B1476">
         <v>2305</v>
@@ -21483,7 +21483,7 @@
     </row>
     <row r="1477" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1477" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B1477">
         <v>2305</v>
@@ -21497,7 +21497,7 @@
     </row>
     <row r="1478" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1478" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B1478">
         <v>2305</v>
@@ -21511,7 +21511,7 @@
     </row>
     <row r="1479" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1479" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B1479">
         <v>2305</v>
@@ -21525,7 +21525,7 @@
     </row>
     <row r="1480" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1480" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B1480">
         <v>2305</v>
@@ -21539,7 +21539,7 @@
     </row>
     <row r="1481" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1481" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B1481">
         <v>2305</v>
@@ -21553,7 +21553,7 @@
     </row>
     <row r="1482" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1482" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B1482">
         <v>2305</v>
@@ -21567,7 +21567,7 @@
     </row>
     <row r="1483" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1483" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B1483">
         <v>2305</v>
@@ -21581,7 +21581,7 @@
     </row>
     <row r="1484" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1484" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B1484">
         <v>2305</v>
@@ -21595,7 +21595,7 @@
     </row>
     <row r="1485" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1485" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B1485">
         <v>2305</v>
@@ -21609,7 +21609,7 @@
     </row>
     <row r="1486" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1486" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B1486">
         <v>2306</v>
@@ -21623,7 +21623,7 @@
     </row>
     <row r="1487" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1487" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B1487">
         <v>2306</v>
@@ -21637,7 +21637,7 @@
     </row>
     <row r="1488" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1488" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B1488">
         <v>2306</v>
@@ -21651,7 +21651,7 @@
     </row>
     <row r="1489" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1489" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B1489">
         <v>2306</v>
@@ -21665,7 +21665,7 @@
     </row>
     <row r="1490" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1490" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B1490">
         <v>2306</v>
@@ -21679,7 +21679,7 @@
     </row>
     <row r="1491" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1491" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B1491">
         <v>2306</v>
@@ -21693,7 +21693,7 @@
     </row>
     <row r="1492" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1492" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B1492">
         <v>2306</v>
@@ -21707,7 +21707,7 @@
     </row>
     <row r="1493" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1493" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B1493">
         <v>2306</v>
@@ -21721,7 +21721,7 @@
     </row>
     <row r="1494" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1494" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B1494">
         <v>2306</v>
@@ -21735,7 +21735,7 @@
     </row>
     <row r="1495" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1495" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B1495">
         <v>2306</v>
@@ -21749,7 +21749,7 @@
     </row>
     <row r="1496" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1496" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B1496">
         <v>2306</v>
@@ -21763,7 +21763,7 @@
     </row>
     <row r="1497" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1497" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B1497">
         <v>2306</v>
@@ -21777,7 +21777,7 @@
     </row>
     <row r="1498" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1498" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B1498">
         <v>2306</v>
@@ -21791,7 +21791,7 @@
     </row>
     <row r="1499" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1499" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B1499">
         <v>2307</v>
@@ -21805,7 +21805,7 @@
     </row>
     <row r="1500" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1500" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B1500">
         <v>2307</v>
@@ -21819,7 +21819,7 @@
     </row>
     <row r="1501" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1501" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B1501">
         <v>2307</v>
@@ -21833,7 +21833,7 @@
     </row>
     <row r="1502" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1502" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B1502">
         <v>2307</v>
@@ -21847,7 +21847,7 @@
     </row>
     <row r="1503" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1503" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B1503">
         <v>2307</v>
@@ -21861,7 +21861,7 @@
     </row>
     <row r="1504" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1504" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B1504">
         <v>2307</v>
@@ -21875,7 +21875,7 @@
     </row>
     <row r="1505" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1505" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B1505">
         <v>2307</v>
@@ -21889,7 +21889,7 @@
     </row>
     <row r="1506" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1506" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B1506">
         <v>2307</v>
@@ -21903,7 +21903,7 @@
     </row>
     <row r="1507" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1507" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B1507">
         <v>2307</v>
@@ -21917,7 +21917,7 @@
     </row>
     <row r="1508" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1508" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B1508">
         <v>2307</v>
@@ -21931,7 +21931,7 @@
     </row>
     <row r="1509" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1509" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B1509">
         <v>2307</v>
@@ -21958,17 +21958,17 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -23095,7 +23095,7 @@
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A107" t="s">
-        <v>105</v>
+        <v>146</v>
       </c>
       <c r="B107">
         <v>1905</v>
@@ -23106,7 +23106,7 @@
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A108" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B108">
         <v>1906</v>
@@ -23117,7 +23117,7 @@
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A109" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B109">
         <v>1907</v>
@@ -23128,7 +23128,7 @@
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A110" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B110">
         <v>1908</v>
@@ -23139,7 +23139,7 @@
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A111" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B111">
         <v>2001</v>
@@ -23150,7 +23150,7 @@
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A112" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B112">
         <v>2002</v>
@@ -23161,7 +23161,7 @@
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A113" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B113">
         <v>2003</v>
@@ -23172,7 +23172,7 @@
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A114" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B114">
         <v>2101</v>
@@ -23183,7 +23183,7 @@
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A115" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B115">
         <v>2102</v>
@@ -23194,7 +23194,7 @@
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A116" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B116">
         <v>2103</v>
@@ -23205,7 +23205,7 @@
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A117" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B117">
         <v>2104</v>
@@ -23216,7 +23216,7 @@
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A118" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B118">
         <v>2105</v>
@@ -23227,7 +23227,7 @@
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A119" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B119">
         <v>2106</v>
@@ -23238,7 +23238,7 @@
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A120" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B120">
         <v>2107</v>
@@ -23249,7 +23249,7 @@
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A121" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B121">
         <v>2108</v>
@@ -23260,7 +23260,7 @@
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A122" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B122">
         <v>2109</v>
@@ -23271,7 +23271,7 @@
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A123" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B123">
         <v>2201</v>
@@ -23282,7 +23282,7 @@
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A124" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B124">
         <v>2202</v>
@@ -23293,7 +23293,7 @@
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A125" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B125">
         <v>2203</v>
@@ -23304,7 +23304,7 @@
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A126" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B126">
         <v>2204</v>
@@ -23315,7 +23315,7 @@
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A127" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B127">
         <v>2205</v>
@@ -23326,7 +23326,7 @@
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A128" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B128">
         <v>2206</v>
@@ -23337,7 +23337,7 @@
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A129" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B129">
         <v>2207</v>
@@ -23348,7 +23348,7 @@
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A130" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B130">
         <v>2208</v>
@@ -23359,7 +23359,7 @@
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A131" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B131">
         <v>2210</v>
@@ -23370,7 +23370,7 @@
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A132" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B132">
         <v>2211</v>
@@ -23381,7 +23381,7 @@
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A133" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B133">
         <v>2212</v>
@@ -23392,7 +23392,7 @@
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A134" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B134">
         <v>2213</v>
@@ -23403,7 +23403,7 @@
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A135" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B135">
         <v>2215</v>
@@ -23414,7 +23414,7 @@
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A136" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B136">
         <v>2301</v>
@@ -23425,7 +23425,7 @@
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A137" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B137">
         <v>2302</v>
@@ -23436,7 +23436,7 @@
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A138" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B138">
         <v>2303</v>
@@ -23447,7 +23447,7 @@
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A139" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B139">
         <v>2304</v>
@@ -23458,7 +23458,7 @@
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A140" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B140">
         <v>2305</v>
@@ -23469,7 +23469,7 @@
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A141" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B141">
         <v>2306</v>
@@ -23480,7 +23480,7 @@
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A142" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B142">
         <v>2307</v>

</xml_diff>